<commit_message>
clusters finais e figuras em inglês
</commit_message>
<xml_diff>
--- a/databases/metricas_avaliacao_clusters.xlsx
+++ b/databases/metricas_avaliacao_clusters.xlsx
@@ -403,22 +403,22 @@
         </is>
       </c>
       <c r="B2">
-        <v>0.7941069971283413</v>
+        <v>0.7921386638930618</v>
       </c>
       <c r="C2">
-        <v>0.9698700015920991</v>
+        <v>0.9656836697298948</v>
       </c>
       <c r="D2">
         <v>0.001594896331738431</v>
       </c>
       <c r="E2">
-        <v>0.6958733253577559</v>
+        <v>0.6962785504213564</v>
       </c>
       <c r="F2">
-        <v>8062.97342540988</v>
+        <v>8109.234314366015</v>
       </c>
       <c r="G2">
-        <v>9633.290544473339</v>
+        <v>9695.03555022506</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -433,22 +433,22 @@
         </is>
       </c>
       <c r="B3">
-        <v>0.7420301852618171</v>
+        <v>0.7409590842431715</v>
       </c>
       <c r="C3">
-        <v>0.852250640736768</v>
+        <v>0.8473853207615423</v>
       </c>
       <c r="D3">
         <v>0.001715265866209264</v>
       </c>
       <c r="E3">
-        <v>0.7111539044691423</v>
+        <v>0.7115145972499541</v>
       </c>
       <c r="F3">
-        <v>10313.28715706212</v>
+        <v>10382.20471462729</v>
       </c>
       <c r="G3">
-        <v>12573.21527936072</v>
+        <v>12675.40697608507</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -463,22 +463,22 @@
         </is>
       </c>
       <c r="B4">
-        <v>0.7336926191776074</v>
+        <v>0.7332471668662663</v>
       </c>
       <c r="C4">
-        <v>0.865662558508083</v>
+        <v>0.860316877404434</v>
       </c>
       <c r="D4">
         <v>0.001766784452296813</v>
       </c>
       <c r="E4">
-        <v>0.7086888294100762</v>
+        <v>0.7090514933228995</v>
       </c>
       <c r="F4">
-        <v>9709.787234853789</v>
+        <v>9782.009177852766</v>
       </c>
       <c r="G4">
-        <v>11610.13017728958</v>
+        <v>11721.80198026232</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -493,22 +493,22 @@
         </is>
       </c>
       <c r="B5">
-        <v>0.7458629981298873</v>
+        <v>0.7424733057440944</v>
       </c>
       <c r="C5">
-        <v>0.9378124923791673</v>
+        <v>0.9341181358009374</v>
       </c>
       <c r="D5">
-        <v>0.001828153564899453</v>
+        <v>0.00181488203266787</v>
       </c>
       <c r="E5">
-        <v>0.7174752056770378</v>
+        <v>0.7168033615433581</v>
       </c>
       <c r="F5">
-        <v>9673.268714747495</v>
+        <v>9412.567879535103</v>
       </c>
       <c r="G5">
-        <v>11314.07875019638</v>
+        <v>10991.33537419847</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -523,22 +523,22 @@
         </is>
       </c>
       <c r="B6">
-        <v>0.748597769168126</v>
+        <v>0.7290653489051589</v>
       </c>
       <c r="C6">
-        <v>0.961271620131613</v>
+        <v>0.9108856787515828</v>
       </c>
       <c r="D6">
-        <v>0.001937984496124024</v>
+        <v>0.001834862385321094</v>
       </c>
       <c r="E6">
-        <v>0.7252054629014772</v>
+        <v>0.7236426044474198</v>
       </c>
       <c r="F6">
-        <v>11260.50430122014</v>
+        <v>8411.112067538839</v>
       </c>
       <c r="G6">
-        <v>13104.23769653571</v>
+        <v>9781.47507323989</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -553,22 +553,22 @@
         </is>
       </c>
       <c r="B7">
-        <v>0.7201452044264669</v>
+        <v>0.7183591274932485</v>
       </c>
       <c r="C7">
-        <v>0.7897485784321021</v>
+        <v>0.7860424993761649</v>
       </c>
       <c r="D7">
         <v>0.001666666666666661</v>
       </c>
       <c r="E7">
-        <v>0.7420467099573532</v>
+        <v>0.7420273857319543</v>
       </c>
       <c r="F7">
-        <v>10281.6413626909</v>
+        <v>10316.50312925316</v>
       </c>
       <c r="G7">
-        <v>10706.96282543698</v>
+        <v>10741.80402207091</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -583,22 +583,22 @@
         </is>
       </c>
       <c r="B8">
-        <v>0.7510915564717757</v>
+        <v>0.7505295310804454</v>
       </c>
       <c r="C8">
-        <v>0.8866966415312879</v>
+        <v>0.8734997492287507</v>
       </c>
       <c r="D8">
-        <v>0.00179856115107913</v>
+        <v>0.001795332136445244</v>
       </c>
       <c r="E8">
-        <v>0.7198038755771549</v>
+        <v>0.7199106460213437</v>
       </c>
       <c r="F8">
-        <v>11685.59996623936</v>
+        <v>11727.42992223991</v>
       </c>
       <c r="G8">
-        <v>13294.55292056119</v>
+        <v>13361.27192016878</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -613,22 +613,22 @@
         </is>
       </c>
       <c r="B9">
-        <v>0.7558855278715617</v>
+        <v>0.7615978523819178</v>
       </c>
       <c r="C9">
-        <v>0.9547006172040674</v>
+        <v>0.942774051430089</v>
       </c>
       <c r="D9">
-        <v>0.002016129032258057</v>
+        <v>0.002004008016032066</v>
       </c>
       <c r="E9">
-        <v>0.7217028898186665</v>
+        <v>0.7216899676452846</v>
       </c>
       <c r="F9">
-        <v>13068.71162041135</v>
+        <v>13023.63781900941</v>
       </c>
       <c r="G9">
-        <v>15077.19029248069</v>
+        <v>15141.52070482313</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -643,22 +643,22 @@
         </is>
       </c>
       <c r="B10">
-        <v>0.5856783331102879</v>
+        <v>0.5825913203616401</v>
       </c>
       <c r="C10">
-        <v>0.6398184129959058</v>
+        <v>0.6376043147213164</v>
       </c>
       <c r="D10">
         <v>0.003984063745019906</v>
       </c>
       <c r="E10">
-        <v>0.7206640131454861</v>
+        <v>0.7204560891611551</v>
       </c>
       <c r="F10">
-        <v>16445.76015979713</v>
+        <v>16587.42630116144</v>
       </c>
       <c r="G10">
-        <v>19138.87196716154</v>
+        <v>19198.94995451903</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -673,22 +673,22 @@
         </is>
       </c>
       <c r="B11">
-        <v>0.5848393160660391</v>
+        <v>0.5825055690645841</v>
       </c>
       <c r="C11">
-        <v>0.6608595957387632</v>
+        <v>0.6536829015094212</v>
       </c>
       <c r="D11">
         <v>0.003984063745019906</v>
       </c>
       <c r="E11">
-        <v>0.7181131935473488</v>
+        <v>0.7182137294561327</v>
       </c>
       <c r="F11">
-        <v>20456.57438916304</v>
+        <v>20636.97660213238</v>
       </c>
       <c r="G11">
-        <v>23523.62330836613</v>
+        <v>23805.65466837364</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="B12">
-        <v>0.7071160891048286</v>
+        <v>0.7053803477032572</v>
       </c>
       <c r="C12">
-        <v>0.7600670576393588</v>
+        <v>0.7564631773331069</v>
       </c>
       <c r="D12">
         <v>0.001680672268907557</v>
       </c>
       <c r="E12">
-        <v>0.7450465831222597</v>
+        <v>0.7449461241127394</v>
       </c>
       <c r="F12">
-        <v>10219.71883090043</v>
+        <v>10246.45050768732</v>
       </c>
       <c r="G12">
-        <v>10343.90999708814</v>
+        <v>10367.36273918394</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -733,22 +733,22 @@
         </is>
       </c>
       <c r="B13">
-        <v>0.7819523670823411</v>
+        <v>0.7800664596414588</v>
       </c>
       <c r="C13">
-        <v>0.9416378409377564</v>
+        <v>0.9363643663653314</v>
       </c>
       <c r="D13">
         <v>0.001680672268907557</v>
       </c>
       <c r="E13">
-        <v>0.6879117916236731</v>
+        <v>0.6883586903922368</v>
       </c>
       <c r="F13">
-        <v>8920.469200580463</v>
+        <v>8985.697260377401</v>
       </c>
       <c r="G13">
-        <v>10805.39101522825</v>
+        <v>10897.55806299406</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -763,22 +763,22 @@
         </is>
       </c>
       <c r="B14">
-        <v>0.748048988778814</v>
+        <v>0.7506189534028507</v>
       </c>
       <c r="C14">
-        <v>0.8991450799132934</v>
+        <v>0.9191916800215086</v>
       </c>
       <c r="D14">
         <v>0.001953124999999993</v>
       </c>
       <c r="E14">
-        <v>0.7100172886641353</v>
+        <v>0.7100629162544673</v>
       </c>
       <c r="F14">
-        <v>12485.30141232235</v>
+        <v>12473.90242804929</v>
       </c>
       <c r="G14">
-        <v>14409.00250696343</v>
+        <v>14311.13603291362</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -793,22 +793,22 @@
         </is>
       </c>
       <c r="B15">
-        <v>0.5683805860633697</v>
+        <v>0.5656024372176113</v>
       </c>
       <c r="C15">
-        <v>0.6323218400591986</v>
+        <v>0.6257846277592742</v>
       </c>
       <c r="D15">
         <v>0.003984063745019906</v>
       </c>
       <c r="E15">
-        <v>0.710149974489791</v>
+        <v>0.7100889731900483</v>
       </c>
       <c r="F15">
-        <v>15575.81885903143</v>
+        <v>15662.34535734599</v>
       </c>
       <c r="G15">
-        <v>17765.40204013872</v>
+        <v>17904.07075757172</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -823,22 +823,22 @@
         </is>
       </c>
       <c r="B16">
-        <v>0.5954961683593516</v>
+        <v>0.5928858433194888</v>
       </c>
       <c r="C16">
-        <v>0.6808177018982697</v>
+        <v>0.6724545072721113</v>
       </c>
       <c r="D16">
         <v>0.003984063745019906</v>
       </c>
       <c r="E16">
-        <v>0.7102923817263634</v>
+        <v>0.7105629453110597</v>
       </c>
       <c r="F16">
-        <v>18145.84483130118</v>
+        <v>18337.79243504147</v>
       </c>
       <c r="G16">
-        <v>20198.72490095205</v>
+        <v>20465.34502241612</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -853,22 +853,22 @@
         </is>
       </c>
       <c r="B17">
-        <v>0.09811726516898804</v>
+        <v>0.09788433563054418</v>
       </c>
       <c r="C17">
-        <v>0.1174139167798748</v>
+        <v>0.1171797793816212</v>
       </c>
       <c r="D17">
         <v>0.3130252100840336</v>
       </c>
       <c r="E17">
-        <v>0.9320719076795019</v>
+        <v>0.9322552304793569</v>
       </c>
       <c r="F17">
-        <v>411.9554488308174</v>
+        <v>414.6981733148527</v>
       </c>
       <c r="G17">
-        <v>352.3978899943585</v>
+        <v>354.5385277928403</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -883,22 +883,22 @@
         </is>
       </c>
       <c r="B18">
-        <v>0.2147727843112944</v>
+        <v>0.2146482440885665</v>
       </c>
       <c r="C18">
-        <v>0.2650556908938559</v>
+        <v>0.2649332763876824</v>
       </c>
       <c r="D18">
         <v>0.3151125401929259</v>
       </c>
       <c r="E18">
-        <v>0.8935053748094735</v>
+        <v>0.8938425208602352</v>
       </c>
       <c r="F18">
-        <v>356.5848766396952</v>
+        <v>359.0953714209782</v>
       </c>
       <c r="G18">
-        <v>307.1517160718903</v>
+        <v>309.1030665340019</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -913,22 +913,22 @@
         </is>
       </c>
       <c r="B19">
-        <v>0.1078960254630286</v>
+        <v>0.1077026866909191</v>
       </c>
       <c r="C19">
-        <v>0.142125283332104</v>
+        <v>0.1419581126004041</v>
       </c>
       <c r="D19">
         <v>0.2122186495176849</v>
       </c>
       <c r="E19">
-        <v>0.8863858590672992</v>
+        <v>0.8867424995401773</v>
       </c>
       <c r="F19">
-        <v>238.3148843262178</v>
+        <v>239.9931130639536</v>
       </c>
       <c r="G19">
-        <v>205.4637953848905</v>
+        <v>206.7695911977547</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -943,22 +943,22 @@
         </is>
       </c>
       <c r="B20">
-        <v>0.0901125458778273</v>
+        <v>0.08979748823712735</v>
       </c>
       <c r="C20">
-        <v>0.09672253883738814</v>
+        <v>0.09641883286624867</v>
       </c>
       <c r="D20">
         <v>0.112540192926045</v>
       </c>
       <c r="E20">
-        <v>0.8861031152109551</v>
+        <v>0.886459704912805</v>
       </c>
       <c r="F20">
-        <v>178.8029098811049</v>
+        <v>180.0621093224045</v>
       </c>
       <c r="G20">
-        <v>154.2247559271684</v>
+        <v>155.2050058160424</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -973,22 +973,22 @@
         </is>
       </c>
       <c r="B21">
-        <v>0.1220961820212341</v>
+        <v>0.1111660533155121</v>
       </c>
       <c r="C21">
-        <v>0.1280274110821686</v>
+        <v>0.1174147798005934</v>
       </c>
       <c r="D21">
-        <v>0.04905660377358493</v>
+        <v>0.04912280701754381</v>
       </c>
       <c r="E21">
-        <v>0.8311822064066956</v>
+        <v>0.838298757762344</v>
       </c>
       <c r="F21">
-        <v>201.1758289251678</v>
+        <v>175.1997006219439</v>
       </c>
       <c r="G21">
-        <v>176.0954538847682</v>
+        <v>152.2744222528795</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1003,22 +1003,22 @@
         </is>
       </c>
       <c r="B22">
-        <v>0.3038224012989404</v>
+        <v>0.3035014612166439</v>
       </c>
       <c r="C22">
-        <v>0.3422118509126172</v>
+        <v>0.3418961777605273</v>
       </c>
       <c r="D22">
         <v>0.3151125401929259</v>
       </c>
       <c r="E22">
-        <v>0.9137829586790857</v>
+        <v>0.914049344840546</v>
       </c>
       <c r="F22">
-        <v>679.052777815384</v>
+        <v>683.8129655465774</v>
       </c>
       <c r="G22">
-        <v>584.6214685171649</v>
+        <v>588.3170937312703</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1033,22 +1033,22 @@
         </is>
       </c>
       <c r="B23">
-        <v>0.4676693607677068</v>
+        <v>0.4413146668735033</v>
       </c>
       <c r="C23">
-        <v>0.5098351411084578</v>
+        <v>0.5099334292151916</v>
       </c>
       <c r="D23">
-        <v>0.003984063745019977</v>
+        <v>0.0199203187250996</v>
       </c>
       <c r="E23">
-        <v>0.7377133860967758</v>
+        <v>0.7896402423141253</v>
       </c>
       <c r="F23">
-        <v>3816.205661906449</v>
+        <v>865.034424258139</v>
       </c>
       <c r="G23">
-        <v>2826.750655711593</v>
+        <v>782.7477138605682</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1063,22 +1063,22 @@
         </is>
       </c>
       <c r="B24">
-        <v>0.3713754821589448</v>
+        <v>0.3035036705526018</v>
       </c>
       <c r="C24">
-        <v>0.4142051405771846</v>
+        <v>0.353742100141515</v>
       </c>
       <c r="D24">
-        <v>0.005050505050505122</v>
+        <v>0.02512562814070352</v>
       </c>
       <c r="E24">
-        <v>0.7372695887299486</v>
+        <v>0.7897301568202093</v>
       </c>
       <c r="F24">
-        <v>2594.95375592819</v>
+        <v>592.2712032302167</v>
       </c>
       <c r="G24">
-        <v>1917.322601716682</v>
+        <v>535.1718334699847</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1093,22 +1093,22 @@
         </is>
       </c>
       <c r="B25">
-        <v>0.380217787654952</v>
+        <v>0.417301610174766</v>
       </c>
       <c r="C25">
-        <v>0.418091645951883</v>
+        <v>0.449286915172545</v>
       </c>
       <c r="D25">
-        <v>0.00877192982456153</v>
+        <v>0.007874015748031539</v>
       </c>
       <c r="E25">
-        <v>0.7205539584925527</v>
+        <v>0.7280126377645855</v>
       </c>
       <c r="F25">
-        <v>2120.719767435529</v>
+        <v>4483.106811983894</v>
       </c>
       <c r="G25">
-        <v>1548.526040890759</v>
+        <v>3915.764066549737</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1123,22 +1123,22 @@
         </is>
       </c>
       <c r="B26">
-        <v>0.4409108665839517</v>
+        <v>0.4741782697889286</v>
       </c>
       <c r="C26">
-        <v>0.4774146083058366</v>
+        <v>0.5156359733455057</v>
       </c>
       <c r="D26">
-        <v>0.008928571428571556</v>
+        <v>0.009345794392523412</v>
       </c>
       <c r="E26">
-        <v>0.6936587588707978</v>
+        <v>0.6908633954396576</v>
       </c>
       <c r="F26">
-        <v>1785.885298581713</v>
+        <v>4507.767724189112</v>
       </c>
       <c r="G26">
-        <v>1296.064717520166</v>
+        <v>3735.380668741548</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -1153,22 +1153,22 @@
         </is>
       </c>
       <c r="B27">
-        <v>0.4686024942304404</v>
+        <v>0.4220732461249934</v>
       </c>
       <c r="C27">
-        <v>0.6638586856928255</v>
+        <v>0.4498079282799691</v>
       </c>
       <c r="D27">
-        <v>0.03403141361256546</v>
+        <v>0.038781163434903</v>
       </c>
       <c r="E27">
-        <v>0.883273379583486</v>
+        <v>0.8962282144145611</v>
       </c>
       <c r="F27">
-        <v>874.8514868835268</v>
+        <v>782.7634117339105</v>
       </c>
       <c r="G27">
-        <v>736.979205489239</v>
+        <v>685.3112220795941</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1183,22 +1183,22 @@
         </is>
       </c>
       <c r="B28">
-        <v>0.3248229198334152</v>
+        <v>0.3125424208524248</v>
       </c>
       <c r="C28">
-        <v>0.3702666044674546</v>
+        <v>0.4185968610906735</v>
       </c>
       <c r="D28">
-        <v>0.04905660377358493</v>
+        <v>0.04912280701754381</v>
       </c>
       <c r="E28">
-        <v>0.8595782764471059</v>
+        <v>0.8723621734205375</v>
       </c>
       <c r="F28">
-        <v>488.8084063085658</v>
+        <v>428.9921101569612</v>
       </c>
       <c r="G28">
-        <v>426.7008752984581</v>
+        <v>370.997349530146</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1213,22 +1213,22 @@
         </is>
       </c>
       <c r="B29">
-        <v>0.2671872146923461</v>
+        <v>0.4332066054843731</v>
       </c>
       <c r="C29">
-        <v>0.3549902737871833</v>
+        <v>0.4960995890416366</v>
       </c>
       <c r="D29">
-        <v>0.04905660377358493</v>
+        <v>0.005649717514124273</v>
       </c>
       <c r="E29">
-        <v>0.831514781250421</v>
+        <v>0.7333631821407731</v>
       </c>
       <c r="F29">
-        <v>334.5748050198121</v>
+        <v>2727.72603995589</v>
       </c>
       <c r="G29">
-        <v>292.5771855591126</v>
+        <v>2014.473508603711</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -1243,22 +1243,22 @@
         </is>
       </c>
       <c r="B30">
-        <v>0.3640603931875296</v>
+        <v>0.3567137252070376</v>
       </c>
       <c r="C30">
-        <v>0.4445158492846142</v>
+        <v>0.4399384965470529</v>
       </c>
       <c r="D30">
-        <v>0.006493506493506471</v>
+        <v>0.005747126436781589</v>
       </c>
       <c r="E30">
-        <v>0.7289342884166479</v>
+        <v>0.7308181288333772</v>
       </c>
       <c r="F30">
-        <v>2113.650591453974</v>
+        <v>2063.861669336371</v>
       </c>
       <c r="G30">
-        <v>1561.259628940038</v>
+        <v>1524.856654985365</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -1273,22 +1273,22 @@
         </is>
       </c>
       <c r="B31">
-        <v>0.4222288091246418</v>
+        <v>0.4127182840288467</v>
       </c>
       <c r="C31">
-        <v>0.4888796032842361</v>
+        <v>0.4955497421433226</v>
       </c>
       <c r="D31">
         <v>0.009090909090909059</v>
       </c>
       <c r="E31">
-        <v>0.6967792540664742</v>
+        <v>0.697028718967043</v>
       </c>
       <c r="F31">
-        <v>1848.602976678229</v>
+        <v>1822.9624769826</v>
       </c>
       <c r="G31">
-        <v>1350.219366201652</v>
+        <v>1330.883666305314</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -1303,22 +1303,22 @@
         </is>
       </c>
       <c r="B32">
-        <v>0.9049234703619804</v>
+        <v>0.736886840792417</v>
       </c>
       <c r="C32">
-        <v>1.041681636072286</v>
+        <v>0.8487221460099431</v>
       </c>
       <c r="D32">
-        <v>0.0006988120195667371</v>
+        <v>0.0023696682464455</v>
       </c>
       <c r="E32">
-        <v>0.70013466432349</v>
+        <v>0.7029715218631571</v>
       </c>
       <c r="F32">
-        <v>6123.458000250968</v>
+        <v>9623.28174705128</v>
       </c>
       <c r="G32">
-        <v>7632.147130635087</v>
+        <v>11687.76161466941</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -1333,22 +1333,22 @@
         </is>
       </c>
       <c r="B33">
-        <v>0.9535457256018541</v>
+        <v>0.7113217099775129</v>
       </c>
       <c r="C33">
-        <v>1.184868294989723</v>
+        <v>0.8589481358715121</v>
       </c>
       <c r="D33">
-        <v>0.000713266761768899</v>
+        <v>0.002544529262086505</v>
       </c>
       <c r="E33">
-        <v>0.6920982455993094</v>
+        <v>0.6959008354590822</v>
       </c>
       <c r="F33">
-        <v>5460.627172271504</v>
+        <v>10904.52828633181</v>
       </c>
       <c r="G33">
-        <v>6635.045792813399</v>
+        <v>12865.49011207762</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -1363,22 +1363,22 @@
         </is>
       </c>
       <c r="B34">
-        <v>1.019854831984265</v>
+        <v>0.6802065453972648</v>
       </c>
       <c r="C34">
-        <v>1.244336291294026</v>
+        <v>0.7764315594395081</v>
       </c>
       <c r="D34">
-        <v>0.000730994152046781</v>
+        <v>0.002777777777777768</v>
       </c>
       <c r="E34">
-        <v>0.71497233248403</v>
+        <v>0.7181804809669858</v>
       </c>
       <c r="F34">
-        <v>5378.266989497894</v>
+        <v>14456.32738843468</v>
       </c>
       <c r="G34">
-        <v>6596.607872991262</v>
+        <v>17376.85254925521</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -1393,22 +1393,22 @@
         </is>
       </c>
       <c r="B35">
-        <v>1.019863312258381</v>
+        <v>0.6566481199221191</v>
       </c>
       <c r="C35">
-        <v>1.312986296750432</v>
+        <v>0.7763998634527414</v>
       </c>
       <c r="D35">
-        <v>0.000734214390602053</v>
+        <v>0.00283286118980169</v>
       </c>
       <c r="E35">
-        <v>0.7286110550287499</v>
+        <v>0.7324891618630752</v>
       </c>
       <c r="F35">
-        <v>4500.739217323573</v>
+        <v>14060.88790553151</v>
       </c>
       <c r="G35">
-        <v>5413.301273467368</v>
+        <v>16360.7820388286</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -1423,22 +1423,22 @@
         </is>
       </c>
       <c r="B36">
-        <v>1.027139916982323</v>
+        <v>0.6551639989051383</v>
       </c>
       <c r="C36">
-        <v>1.316703728187518</v>
+        <v>0.7570742392944146</v>
       </c>
       <c r="D36">
-        <v>0.00073691967575534</v>
+        <v>0.002873563218390795</v>
       </c>
       <c r="E36">
-        <v>0.7264119403618997</v>
+        <v>0.7304736748153263</v>
       </c>
       <c r="F36">
-        <v>3802.781843884292</v>
+        <v>12959.05706060579</v>
       </c>
       <c r="G36">
-        <v>4579.8531677764</v>
+        <v>15106.32848321054</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -1453,22 +1453,22 @@
         </is>
       </c>
       <c r="B37">
-        <v>0.8762255830828987</v>
+        <v>0.6781948623192956</v>
       </c>
       <c r="C37">
-        <v>0.976179704749904</v>
+        <v>0.7557034301558642</v>
       </c>
       <c r="D37">
-        <v>0.0007092198581560258</v>
+        <v>0.002481389578163763</v>
       </c>
       <c r="E37">
-        <v>0.7377110269737708</v>
+        <v>0.7372061701986623</v>
       </c>
       <c r="F37">
-        <v>7238.86083245517</v>
+        <v>11756.34439918427</v>
       </c>
       <c r="G37">
-        <v>7916.693079840804</v>
+        <v>12277.61144612404</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -1483,22 +1483,22 @@
         </is>
       </c>
       <c r="B38">
-        <v>1.027577622559291</v>
+        <v>0.6846017146411268</v>
       </c>
       <c r="C38">
-        <v>1.240714838713058</v>
+        <v>0.7726216946689727</v>
       </c>
       <c r="D38">
-        <v>0.000734214390602053</v>
+        <v>0.002785515320334252</v>
       </c>
       <c r="E38">
-        <v>0.7197222043785027</v>
+        <v>0.7202623884242696</v>
       </c>
       <c r="F38">
-        <v>6687.422831874392</v>
+        <v>14486.93918221869</v>
       </c>
       <c r="G38">
-        <v>7826.687995502895</v>
+        <v>16585.90919754051</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -1513,22 +1513,22 @@
         </is>
       </c>
       <c r="B39">
-        <v>0.5215189301546734</v>
+        <v>0.6824325418959341</v>
       </c>
       <c r="C39">
-        <v>0.5877699813908108</v>
+        <v>0.7598439720150727</v>
       </c>
       <c r="D39">
-        <v>0.002785515320334252</v>
+        <v>0.003003003003002993</v>
       </c>
       <c r="E39">
-        <v>0.7201330774030085</v>
+        <v>0.7145599096469799</v>
       </c>
       <c r="F39">
-        <v>12422.49192441842</v>
+        <v>16558.11155172021</v>
       </c>
       <c r="G39">
-        <v>13611.03443385328</v>
+        <v>19649.53885117804</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -1543,22 +1543,22 @@
         </is>
       </c>
       <c r="B40">
-        <v>0.5534747945606643</v>
+        <v>0.658778723076003</v>
       </c>
       <c r="C40">
-        <v>0.6179731711939276</v>
+        <v>0.7359986490055449</v>
       </c>
       <c r="D40">
-        <v>0.003012048192771073</v>
+        <v>0.003508771929824549</v>
       </c>
       <c r="E40">
-        <v>0.7134993799018865</v>
+        <v>0.7217047387325027</v>
       </c>
       <c r="F40">
-        <v>15767.92587679735</v>
+        <v>19516.47709665524</v>
       </c>
       <c r="G40">
-        <v>17913.65254074024</v>
+        <v>23398.16331538567</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -1573,22 +1573,22 @@
         </is>
       </c>
       <c r="B41">
-        <v>0.5600227321950216</v>
+        <v>0.5512327232302353</v>
       </c>
       <c r="C41">
-        <v>0.6379719877295922</v>
+        <v>0.5868856623665393</v>
       </c>
       <c r="D41">
-        <v>0.003546099290780129</v>
+        <v>0.007692307692307665</v>
       </c>
       <c r="E41">
-        <v>0.7178449057149298</v>
+        <v>0.7169432770638344</v>
       </c>
       <c r="F41">
-        <v>19621.23806605646</v>
+        <v>21207.63932174511</v>
       </c>
       <c r="G41">
-        <v>22380.76968647008</v>
+        <v>25078.42998510876</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -1603,22 +1603,22 @@
         </is>
       </c>
       <c r="B42">
-        <v>0.8922701130224272</v>
+        <v>0.7134406505264346</v>
       </c>
       <c r="C42">
-        <v>0.9979619707292152</v>
+        <v>0.799248723381678</v>
       </c>
       <c r="D42">
-        <v>0.0007022471910112366</v>
+        <v>0.002409638554216869</v>
       </c>
       <c r="E42">
-        <v>0.7204330360227654</v>
+        <v>0.7225210359168457</v>
       </c>
       <c r="F42">
-        <v>6737.899100096522</v>
+        <v>10846.11350518746</v>
       </c>
       <c r="G42">
-        <v>8131.312888958292</v>
+        <v>12622.98257650499</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -1633,22 +1633,22 @@
         </is>
       </c>
       <c r="B43">
-        <v>0.4856166948147464</v>
+        <v>0.6871910623288846</v>
       </c>
       <c r="C43">
-        <v>0.5430704102738293</v>
+        <v>0.8015858605684043</v>
       </c>
       <c r="D43">
-        <v>0.002409638554216869</v>
+        <v>0.002840909090909081</v>
       </c>
       <c r="E43">
-        <v>0.7223913193933418</v>
+        <v>0.7143821807716456</v>
       </c>
       <c r="F43">
-        <v>7393.587079901004</v>
+        <v>13930.85916346719</v>
       </c>
       <c r="G43">
-        <v>8110.232734417499</v>
+        <v>14734.69793514511</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -1663,22 +1663,22 @@
         </is>
       </c>
       <c r="B44">
-        <v>0.5236126791985455</v>
+        <v>0.6582978390153964</v>
       </c>
       <c r="C44">
-        <v>0.6097292969379284</v>
+        <v>0.7538547222873255</v>
       </c>
       <c r="D44">
         <v>0.002840909090909081</v>
       </c>
       <c r="E44">
-        <v>0.7142539254429613</v>
+        <v>0.7139115482460222</v>
       </c>
       <c r="F44">
-        <v>11962.75589099706</v>
+        <v>13968.58755480741</v>
       </c>
       <c r="G44">
-        <v>12132.81416305967</v>
+        <v>16654.1820505789</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -1693,22 +1693,22 @@
         </is>
       </c>
       <c r="B45">
-        <v>0.5332137771738227</v>
+        <v>0.6358525921130131</v>
       </c>
       <c r="C45">
-        <v>0.6099156990391607</v>
+        <v>0.7143531506955415</v>
       </c>
       <c r="D45">
-        <v>0.002840909090909081</v>
+        <v>0.003984063745019906</v>
       </c>
       <c r="E45">
-        <v>0.7137833774115077</v>
+        <v>0.7142572578734309</v>
       </c>
       <c r="F45">
-        <v>13326.06994153478</v>
+        <v>16204.60188063511</v>
       </c>
       <c r="G45">
-        <v>15236.09542572822</v>
+        <v>19572.14641796598</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -1723,22 +1723,22 @@
         </is>
       </c>
       <c r="B46">
-        <v>0.5389952811595231</v>
+        <v>0.6204771216272738</v>
       </c>
       <c r="C46">
-        <v>0.6047811784862009</v>
+        <v>0.6965926878202804</v>
       </c>
       <c r="D46">
         <v>0.003984063745019906</v>
       </c>
       <c r="E46">
-        <v>0.7141290249725558</v>
+        <v>0.7157880464469657</v>
       </c>
       <c r="F46">
-        <v>16343.67807830212</v>
+        <v>20013.00933808149</v>
       </c>
       <c r="G46">
-        <v>18974.46844145542</v>
+        <v>23618.55460364598</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -1753,22 +1753,22 @@
         </is>
       </c>
       <c r="B47">
-        <v>0.02734395492110341</v>
+        <v>0.1944555828724138</v>
       </c>
       <c r="C47">
-        <v>0.0301320142340732</v>
+        <v>0.1972060368705121</v>
       </c>
       <c r="D47">
-        <v>2.222466960352423</v>
+        <v>0.3129496402877697</v>
       </c>
       <c r="E47">
-        <v>0.9741233734636061</v>
+        <v>0.8996171603008141</v>
       </c>
       <c r="F47">
-        <v>1336.969108143822</v>
+        <v>314.9722688304263</v>
       </c>
       <c r="G47">
-        <v>1101.198676812705</v>
+        <v>152.3469528024018</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -1783,22 +1783,22 @@
         </is>
       </c>
       <c r="B48">
-        <v>0.1417458781056221</v>
+        <v>0.4199349726989943</v>
       </c>
       <c r="C48">
-        <v>0.1447682102021204</v>
+        <v>0.4440008878179534</v>
       </c>
       <c r="D48">
-        <v>0.3129496402877697</v>
+        <v>0.005681818181818161</v>
       </c>
       <c r="E48">
-        <v>0.8994556491409755</v>
+        <v>0.7306299642706362</v>
       </c>
       <c r="F48">
-        <v>863.6656619282259</v>
+        <v>3356.603885828662</v>
       </c>
       <c r="G48">
-        <v>641.7389664028875</v>
+        <v>2399.54328809959</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -1813,22 +1813,22 @@
         </is>
       </c>
       <c r="B49">
-        <v>0.3240328466672554</v>
+        <v>0.3244095495721811</v>
       </c>
       <c r="C49">
-        <v>0.3429738050797994</v>
+        <v>0.353522358727914</v>
       </c>
       <c r="D49">
         <v>0.005681818181818161</v>
       </c>
       <c r="E49">
-        <v>0.7304987919251658</v>
+        <v>0.7297262685431969</v>
       </c>
       <c r="F49">
-        <v>3220.549708798693</v>
+        <v>2241.649309419259</v>
       </c>
       <c r="G49">
-        <v>2283.006087107082</v>
+        <v>1602.181549796662</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -1843,22 +1843,22 @@
         </is>
       </c>
       <c r="B50">
-        <v>0.2646621464619882</v>
+        <v>0.3908722140598032</v>
       </c>
       <c r="C50">
-        <v>0.2882259820673069</v>
+        <v>0.422231254888875</v>
       </c>
       <c r="D50">
-        <v>0.005681818181818161</v>
+        <v>0.008849557522123862</v>
       </c>
       <c r="E50">
-        <v>0.7295952584411245</v>
+        <v>0.692745293040823</v>
       </c>
       <c r="F50">
-        <v>2418.992043162541</v>
+        <v>1885.588085949523</v>
       </c>
       <c r="G50">
-        <v>1714.43839135307</v>
+        <v>1336.099914482956</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -1873,22 +1873,22 @@
         </is>
       </c>
       <c r="B51">
-        <v>0.3294749126418805</v>
+        <v>0.3865922345321002</v>
       </c>
       <c r="C51">
-        <v>0.3557544732697349</v>
+        <v>0.4179480401624628</v>
       </c>
       <c r="D51">
-        <v>0.008849557522123862</v>
+        <v>0.009900990099009866</v>
       </c>
       <c r="E51">
-        <v>0.6926209222521263</v>
+        <v>0.6887244479945146</v>
       </c>
       <c r="F51">
-        <v>2137.880964596774</v>
+        <v>1530.789064268309</v>
       </c>
       <c r="G51">
-        <v>1500.356773161749</v>
+        <v>1082.575943689808</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -1903,22 +1903,22 @@
         </is>
       </c>
       <c r="B52">
-        <v>0.02734395492110341</v>
+        <v>0.1944555828724138</v>
       </c>
       <c r="C52">
-        <v>0.0301320142340732</v>
+        <v>0.1972060368705121</v>
       </c>
       <c r="D52">
-        <v>2.222466960352423</v>
+        <v>0.3129496402877697</v>
       </c>
       <c r="E52">
-        <v>0.9741233734636061</v>
+        <v>0.8996171603008141</v>
       </c>
       <c r="F52">
-        <v>1336.969108143822</v>
+        <v>314.9722688304263</v>
       </c>
       <c r="G52">
-        <v>1101.198676812705</v>
+        <v>152.3469528024018</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -1933,22 +1933,22 @@
         </is>
       </c>
       <c r="B53">
-        <v>0.1417458781056221</v>
+        <v>0.1280242504754841</v>
       </c>
       <c r="C53">
-        <v>0.1447682102021204</v>
+        <v>0.1544107498334182</v>
       </c>
       <c r="D53">
-        <v>0.3129496402877697</v>
+        <v>0.2446043165467625</v>
       </c>
       <c r="E53">
-        <v>0.8994556491409755</v>
+        <v>0.8816930288426401</v>
       </c>
       <c r="F53">
-        <v>863.6656619282259</v>
+        <v>158.9420820861596</v>
       </c>
       <c r="G53">
-        <v>641.7389664028875</v>
+        <v>77.42575655175156</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -1963,22 +1963,22 @@
         </is>
       </c>
       <c r="B54">
-        <v>0.1026676759565925</v>
+        <v>0.1020427306378295</v>
       </c>
       <c r="C54">
-        <v>0.1232351628910585</v>
+        <v>0.1095776443357989</v>
       </c>
       <c r="D54">
-        <v>0.2446043165467625</v>
+        <v>0.07553956834532378</v>
       </c>
       <c r="E54">
-        <v>0.881534735659724</v>
+        <v>0.8814317213521734</v>
       </c>
       <c r="F54">
-        <v>576.9007656553219</v>
+        <v>105.995479033884</v>
       </c>
       <c r="G54">
-        <v>428.7600180454888</v>
+        <v>51.6884135543381</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -1993,22 +1993,22 @@
         </is>
       </c>
       <c r="B55">
-        <v>0.08695377499024713</v>
+        <v>0.1191798362625988</v>
       </c>
       <c r="C55">
-        <v>0.09360379588143498</v>
+        <v>0.1266204370581611</v>
       </c>
       <c r="D55">
-        <v>0.07553956834532378</v>
+        <v>0.06923076923076926</v>
       </c>
       <c r="E55">
-        <v>0.8812734750826309</v>
+        <v>0.8335933526060766</v>
       </c>
       <c r="F55">
-        <v>432.6472526857038</v>
+        <v>91.10913477934641</v>
       </c>
       <c r="G55">
-        <v>321.5845696081233</v>
+        <v>49.03671481099833</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -2023,22 +2023,22 @@
         </is>
       </c>
       <c r="B56">
-        <v>0.1037323573996905</v>
+        <v>0.1647335323754312</v>
       </c>
       <c r="C56">
-        <v>0.110451174069675</v>
+        <v>0.1682158060800221</v>
       </c>
       <c r="D56">
-        <v>0.06923076923076926</v>
+        <v>0.03404255319148939</v>
       </c>
       <c r="E56">
-        <v>0.8334436949126105</v>
+        <v>0.8138553566622707</v>
       </c>
       <c r="F56">
-        <v>357.5904871478671</v>
+        <v>112.0180261020748</v>
       </c>
       <c r="G56">
-        <v>267.0693897958657</v>
+        <v>74.25386650182591</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -2053,22 +2053,22 @@
         </is>
       </c>
       <c r="B57">
-        <v>0.02734395492110341</v>
+        <v>0.1944555828724138</v>
       </c>
       <c r="C57">
-        <v>0.0301320142340732</v>
+        <v>0.1972060368705121</v>
       </c>
       <c r="D57">
-        <v>2.222466960352423</v>
+        <v>0.3129496402877697</v>
       </c>
       <c r="E57">
-        <v>0.9741233734636061</v>
+        <v>0.8996171603008141</v>
       </c>
       <c r="F57">
-        <v>1336.969108143822</v>
+        <v>314.9722688304263</v>
       </c>
       <c r="G57">
-        <v>1101.198676812705</v>
+        <v>152.3469528024018</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -2083,22 +2083,22 @@
         </is>
       </c>
       <c r="B58">
-        <v>0.1417458781056221</v>
+        <v>0.4141160518221578</v>
       </c>
       <c r="C58">
-        <v>0.1447682102021204</v>
+        <v>0.4270916605904978</v>
       </c>
       <c r="D58">
-        <v>0.3129496402877697</v>
+        <v>0.005882352941176554</v>
       </c>
       <c r="E58">
-        <v>0.8994556491409755</v>
+        <v>0.7310380474646212</v>
       </c>
       <c r="F58">
-        <v>863.6656619282259</v>
+        <v>2999.652668049377</v>
       </c>
       <c r="G58">
-        <v>641.7389664028875</v>
+        <v>2093.345443730012</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -2113,22 +2113,22 @@
         </is>
       </c>
       <c r="B59">
-        <v>0.3196686560096281</v>
+        <v>0.4494502312709366</v>
       </c>
       <c r="C59">
-        <v>0.3302918846592076</v>
+        <v>0.4576044455780459</v>
       </c>
       <c r="D59">
-        <v>0.005882352941176554</v>
+        <v>0.009345794392523497</v>
       </c>
       <c r="E59">
-        <v>0.7309068018546634</v>
+        <v>0.7003044013913833</v>
       </c>
       <c r="F59">
-        <v>2925.442293583142</v>
+        <v>2201.283027972432</v>
       </c>
       <c r="G59">
-        <v>2038.502464200893</v>
+        <v>1519.520657862692</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -2143,22 +2143,22 @@
         </is>
       </c>
       <c r="B60">
-        <v>0.366825478731157</v>
+        <v>0.4964152368348642</v>
       </c>
       <c r="C60">
-        <v>0.3740620678355041</v>
+        <v>0.5170670019461072</v>
       </c>
       <c r="D60">
-        <v>0.009345794392523497</v>
+        <v>0.01052631578947374</v>
       </c>
       <c r="E60">
-        <v>0.7001786734916721</v>
+        <v>0.6871361893500151</v>
       </c>
       <c r="F60">
-        <v>2381.447872041719</v>
+        <v>7647.375165542444</v>
       </c>
       <c r="G60">
-        <v>1640.181668412582</v>
+        <v>6785.959553568397</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
@@ -2173,22 +2173,22 @@
         </is>
       </c>
       <c r="B61">
-        <v>0.4197337754577266</v>
+        <v>0.5030900087191345</v>
       </c>
       <c r="C61">
-        <v>0.4375379277659789</v>
+        <v>0.5242080735752424</v>
       </c>
       <c r="D61">
-        <v>0.01052631578947374</v>
+        <v>0.01123595505617984</v>
       </c>
       <c r="E61">
-        <v>0.6870128255817296</v>
+        <v>0.6852201477110609</v>
       </c>
       <c r="F61">
-        <v>7854.111107167368</v>
+        <v>6190.801521584344</v>
       </c>
       <c r="G61">
-        <v>6722.511470547322</v>
+        <v>5474.545469076982</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>

</xml_diff>